<commit_message>
Дашборд 08.10: +9562 +7044, курс НБУ 50.16/44.86, Hub
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прострочені" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$104</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -519,7 +519,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Дані: 07.10.2026 · без проєктів на паузі/втрачених</t>
+          <t>Дані: 08.10.2026 · без проєктів на паузі/втрачених</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K105"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4603,31 +4603,31 @@
     </row>
     <row r="90">
       <c r="A90" s="8" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="B90" s="9" t="n">
-        <v>6024</v>
+        <v>9562</v>
       </c>
       <c r="C90" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ с. Липовиця Черніг. обл. Модулекс</t>
+          <t>26  SOLAR Наземні СЕС Київ  шт. 0 шт. 0.77 Мвт SolarWind</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Іщук</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Авансовий платіж</t>
         </is>
       </c>
       <c r="F90" s="10" t="n">
-        <v>246402</v>
+        <v>397353.6</v>
       </c>
       <c r="G90" s="10" t="n">
-        <v>0</v>
+        <v>397353.6</v>
       </c>
       <c r="H90" s="11">
         <f>F90-G90</f>
@@ -4635,7 +4635,7 @@
       </c>
       <c r="I90" s="9" t="inlineStr">
         <is>
-          <t>прострочено</t>
+          <t>отримано</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4647,14 +4647,14 @@
     </row>
     <row r="91">
       <c r="A91" s="8" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="B91" s="9" t="n">
-        <v>6024</v>
+        <v>4766</v>
       </c>
       <c r="C91" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ с. Липовиця Черніг. обл. Модулекс</t>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
         </is>
       </c>
       <c r="D91" s="9" t="inlineStr">
@@ -4664,11 +4664,11 @@
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F91" s="10" t="n">
-        <v>3999</v>
+        <v>1263447.42</v>
       </c>
       <c r="G91" s="10" t="n">
         <v>0</v>
@@ -4691,14 +4691,14 @@
     </row>
     <row r="92">
       <c r="A92" s="8" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="B92" s="9" t="n">
-        <v>7244</v>
+        <v>6024</v>
       </c>
       <c r="C92" s="9" t="inlineStr">
         <is>
-          <t>В Модулекс модульна будівля Чернігів</t>
+          <t>-26 ГШ с. Липовиця Черніг. обл. Модулекс</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F92" s="10" t="n">
-        <v>132708.6</v>
+        <v>246402</v>
       </c>
       <c r="G92" s="10" t="n">
         <v>0</v>
@@ -4738,11 +4738,11 @@
         <v>46303</v>
       </c>
       <c r="B93" s="9" t="n">
-        <v>4766</v>
+        <v>6024</v>
       </c>
       <c r="C93" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>-26 ГШ с. Липовиця Черніг. обл. Модулекс</t>
         </is>
       </c>
       <c r="D93" s="9" t="inlineStr">
@@ -4752,11 +4752,11 @@
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F93" s="10" t="n">
-        <v>1263447.42</v>
+        <v>3999</v>
       </c>
       <c r="G93" s="10" t="n">
         <v>0</v>
@@ -4767,7 +4767,7 @@
       </c>
       <c r="I93" s="9" t="inlineStr">
         <is>
-          <t>очікується</t>
+          <t>прострочено</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4779,31 +4779,31 @@
     </row>
     <row r="94">
       <c r="A94" s="8" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="B94" s="9" t="n">
-        <v>5910</v>
+        <v>7244</v>
       </c>
       <c r="C94" s="9" t="inlineStr">
         <is>
-          <t>SGM Brdovec, Хорватия</t>
+          <t>В Модулекс модульна будівля Чернігів</t>
         </is>
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж 60%</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F94" s="10" t="n">
-        <v>17297208.56</v>
+        <v>132708.6</v>
       </c>
       <c r="G94" s="10" t="n">
-        <v>16036852.56</v>
+        <v>0</v>
       </c>
       <c r="H94" s="11">
         <f>F94-G94</f>
@@ -4811,7 +4811,7 @@
       </c>
       <c r="I94" s="9" t="inlineStr">
         <is>
-          <t>очікується</t>
+          <t>прострочено</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4819,11 +4819,7 @@
           <t>2026-10</t>
         </is>
       </c>
-      <c r="K94" s="12" t="inlineStr">
-        <is>
-          <t>€334 181</t>
-        </is>
-      </c>
+      <c r="K94" s="12" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="8" t="n">
@@ -4844,14 +4840,14 @@
       </c>
       <c r="E95" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж 60%</t>
         </is>
       </c>
       <c r="F95" s="10" t="n">
-        <v>2882721.44</v>
+        <v>17297208.56</v>
       </c>
       <c r="G95" s="10" t="n">
-        <v>1374797.36</v>
+        <v>16036852.56</v>
       </c>
       <c r="H95" s="11">
         <f>F95-G95</f>
@@ -4869,37 +4865,37 @@
       </c>
       <c r="K95" s="12" t="inlineStr">
         <is>
-          <t>€55 694</t>
+          <t>€334 181</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="8" t="n">
-        <v>46309</v>
+        <v>46304</v>
       </c>
       <c r="B96" s="9" t="n">
-        <v>7414</v>
+        <v>5910</v>
       </c>
       <c r="C96" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ Фундамент домобудування Володимир</t>
+          <t>SGM Brdovec, Хорватия</t>
         </is>
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F96" s="10" t="n">
-        <v>50822.46</v>
+        <v>2882721.44</v>
       </c>
       <c r="G96" s="10" t="n">
-        <v>0</v>
+        <v>1374797.36</v>
       </c>
       <c r="H96" s="11">
         <f>F96-G96</f>
@@ -4915,32 +4911,36 @@
           <t>2026-10</t>
         </is>
       </c>
-      <c r="K96" s="12" t="inlineStr"/>
+      <c r="K96" s="12" t="inlineStr">
+        <is>
+          <t>€55 694</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B97" s="9" t="n">
-        <v>6352</v>
+        <v>7414</v>
       </c>
       <c r="C97" s="9" t="inlineStr">
         <is>
-          <t>АБМК SCP Blade 8PS</t>
+          <t>-26 ГШ Фундамент домобудування Володимир</t>
         </is>
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F97" s="10" t="n">
-        <v>1119237.26</v>
+        <v>50822.46</v>
       </c>
       <c r="G97" s="10" t="n">
         <v>0</v>
@@ -4980,11 +4980,11 @@
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F98" s="10" t="n">
-        <v>371982.96</v>
+        <v>1119237.26</v>
       </c>
       <c r="G98" s="10" t="n">
         <v>0</v>
@@ -5007,28 +5007,28 @@
     </row>
     <row r="99">
       <c r="A99" s="8" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="B99" s="9" t="n">
-        <v>8497</v>
+        <v>6352</v>
       </c>
       <c r="C99" s="9" t="inlineStr">
         <is>
-          <t>LSG 110MWt   50 points</t>
+          <t>АБМК SCP Blade 8PS</t>
         </is>
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>Іщук</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F99" s="10" t="n">
-        <v>521482</v>
+        <v>371982.96</v>
       </c>
       <c r="G99" s="10" t="n">
         <v>0</v>
@@ -5047,27 +5047,23 @@
           <t>2026-10</t>
         </is>
       </c>
-      <c r="K99" s="12" t="inlineStr">
-        <is>
-          <t>€10 075</t>
-        </is>
-      </c>
+      <c r="K99" s="12" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="8" t="n">
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="B100" s="9" t="n">
-        <v>6356</v>
+        <v>8497</v>
       </c>
       <c r="C100" s="9" t="inlineStr">
         <is>
-          <t>-26 SOLAR Наземні СЕС 3 Kirill Trokhin</t>
+          <t>LSG 110MWt   50 points</t>
         </is>
       </c>
       <c r="D100" s="9" t="inlineStr">
         <is>
-          <t>Хома</t>
+          <t>Іщук</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
@@ -5076,7 +5072,7 @@
         </is>
       </c>
       <c r="F100" s="10" t="n">
-        <v>3325062.4</v>
+        <v>521482</v>
       </c>
       <c r="G100" s="10" t="n">
         <v>0</v>
@@ -5097,34 +5093,34 @@
       </c>
       <c r="K100" s="12" t="inlineStr">
         <is>
-          <t>€64 240</t>
+          <t>€10 075</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="n">
-        <v>46321</v>
+        <v>46316</v>
       </c>
       <c r="B101" s="9" t="n">
-        <v>6352</v>
+        <v>6356</v>
       </c>
       <c r="C101" s="9" t="inlineStr">
         <is>
-          <t>АБМК SCP Blade 8PS</t>
+          <t>-26 SOLAR Наземні СЕС 3 Kirill Trokhin</t>
         </is>
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Хома</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F101" s="10" t="n">
-        <v>651792.28</v>
+        <v>3325062.4</v>
       </c>
       <c r="G101" s="10" t="n">
         <v>0</v>
@@ -5143,32 +5139,36 @@
           <t>2026-10</t>
         </is>
       </c>
-      <c r="K101" s="12" t="inlineStr"/>
+      <c r="K101" s="12" t="inlineStr">
+        <is>
+          <t>€64 240</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="8" t="n">
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="B102" s="9" t="n">
-        <v>6356</v>
+        <v>6352</v>
       </c>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>-26 SOLAR Наземні СЕС 3 Kirill Trokhin</t>
+          <t>АБМК SCP Blade 8PS</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>Хома</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F102" s="10" t="n">
-        <v>665012.48</v>
+        <v>651792.28</v>
       </c>
       <c r="G102" s="10" t="n">
         <v>0</v>
@@ -5187,36 +5187,32 @@
           <t>2026-10</t>
         </is>
       </c>
-      <c r="K102" s="12" t="inlineStr">
-        <is>
-          <t>€12 848</t>
-        </is>
-      </c>
+      <c r="K102" s="12" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="8" t="n">
         <v>46322</v>
       </c>
       <c r="B103" s="9" t="n">
-        <v>7894</v>
+        <v>6356</v>
       </c>
       <c r="C103" s="9" t="inlineStr">
         <is>
-          <t>SCP Фора  Хотів</t>
+          <t>-26 SOLAR Наземні СЕС 3 Kirill Trokhin</t>
         </is>
       </c>
       <c r="D103" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Хома</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F103" s="10" t="n">
-        <v>737597.4</v>
+        <v>665012.48</v>
       </c>
       <c r="G103" s="10" t="n">
         <v>0</v>
@@ -5235,32 +5231,36 @@
           <t>2026-10</t>
         </is>
       </c>
-      <c r="K103" s="12" t="inlineStr"/>
+      <c r="K103" s="12" t="inlineStr">
+        <is>
+          <t>€12 848</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="8" t="n">
-        <v>46330</v>
+        <v>46322</v>
       </c>
       <c r="B104" s="9" t="n">
-        <v>7508</v>
+        <v>7894</v>
       </c>
       <c r="C104" s="9" t="inlineStr">
         <is>
-          <t>8602 Євген Весільна тераса Подорожнє</t>
+          <t>SCP Фора  Хотів</t>
         </is>
       </c>
       <c r="D104" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E104" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F104" s="10" t="n">
-        <v>750999.9399999999</v>
+        <v>737597.4</v>
       </c>
       <c r="G104" s="10" t="n">
         <v>0</v>
@@ -5276,32 +5276,76 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="K104" s="12" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="n">
+        <v>46330</v>
+      </c>
+      <c r="B105" s="9" t="n">
+        <v>7508</v>
+      </c>
+      <c r="C105" s="9" t="inlineStr">
+        <is>
+          <t>8602 Євген Весільна тераса Подорожнє</t>
+        </is>
+      </c>
+      <c r="D105" s="9" t="inlineStr">
+        <is>
+          <t>Заянчковський</t>
+        </is>
+      </c>
+      <c r="E105" s="9" t="inlineStr">
+        <is>
+          <t>Третій платіж</t>
+        </is>
+      </c>
+      <c r="F105" s="10" t="n">
+        <v>750999.9399999999</v>
+      </c>
+      <c r="G105" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" s="11">
+        <f>F105-G105</f>
+        <v/>
+      </c>
+      <c r="I105" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
           <t>2026-11</t>
         </is>
       </c>
-      <c r="K104" s="12" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="E105" s="3" t="inlineStr">
+      <c r="K105" s="12" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="E106" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="F105" s="13">
-        <f>SUM(F2:F104)</f>
-        <v/>
-      </c>
-      <c r="G105" s="13">
-        <f>SUM(G2:G104)</f>
-        <v/>
-      </c>
-      <c r="H105" s="13">
-        <f>SUM(H2:H104)</f>
+      <c r="F106" s="13">
+        <f>SUM(F2:F105)</f>
+        <v/>
+      </c>
+      <c r="G106" s="13">
+        <f>SUM(G2:G105)</f>
+        <v/>
+      </c>
+      <c r="H106" s="13">
+        <f>SUM(H2:H105)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I104"/>
+  <autoFilter ref="A1:I105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5567,7 +5611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5618,23 +5662,23 @@
     </row>
     <row r="2">
       <c r="A2" s="8" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="B2" s="9" t="n">
-        <v>6024</v>
+        <v>4766</v>
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ с. Липовиця Черніг. обл. Модулекс</t>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="E2" s="11" t="n">
-        <v>246402</v>
+        <v>1263447.42</v>
       </c>
       <c r="F2" s="11" t="n">
         <v>0</v>
@@ -5646,23 +5690,23 @@
     </row>
     <row r="3">
       <c r="A3" s="8" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="B3" s="9" t="n">
-        <v>7244</v>
+        <v>6024</v>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>В Модулекс модульна будівля Чернігів</t>
+          <t>-26 ГШ с. Липовиця Черніг. обл. Модулекс</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>132708.6</v>
+        <v>246402</v>
       </c>
       <c r="F3" s="11" t="n">
         <v>0</v>
@@ -5674,26 +5718,26 @@
     </row>
     <row r="4">
       <c r="A4" s="8" t="n">
-        <v>46260</v>
+        <v>46303</v>
       </c>
       <c r="B4" s="9" t="n">
-        <v>6406</v>
+        <v>7244</v>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Максим Яловий Чинадієво</t>
+          <t>В Модулекс модульна будівля Чернігів</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>218602</v>
+        <v>132708.6</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>170788</v>
+        <v>0</v>
       </c>
       <c r="G4" s="11">
         <f>E4-F4</f>
@@ -5702,26 +5746,26 @@
     </row>
     <row r="5">
       <c r="A5" s="8" t="n">
-        <v>46301</v>
+        <v>46260</v>
       </c>
       <c r="B5" s="9" t="n">
-        <v>6024</v>
+        <v>6406</v>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ с. Липовиця Черніг. обл. Модулекс</t>
+          <t>Максим Яловий Чинадієво</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>3999</v>
+        <v>218602</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>0</v>
+        <v>170788</v>
       </c>
       <c r="G5" s="11">
         <f>E5-F5</f>
@@ -5729,26 +5773,54 @@
       </c>
     </row>
     <row r="6">
-      <c r="D6" s="3" t="inlineStr">
+      <c r="A6" s="8" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>6024</v>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>-26 ГШ с. Липовиця Черніг. обл. Модулекс</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Третій платіж</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>3999</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="11">
+        <f>E6-F6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="E6" s="13">
-        <f>SUM(E2:E5)</f>
-        <v/>
-      </c>
-      <c r="F6" s="13">
-        <f>SUM(F2:F5)</f>
-        <v/>
-      </c>
-      <c r="G6" s="13">
-        <f>SUM(G2:G5)</f>
+      <c r="E7" s="13">
+        <f>SUM(E2:E6)</f>
+        <v/>
+      </c>
+      <c r="F7" s="13">
+        <f>SUM(F2:F6)</f>
+        <v/>
+      </c>
+      <c r="G7" s="13">
+        <f>SUM(G2:G6)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G5"/>
+  <autoFilter ref="A1:G6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>